<commit_message>
feat(engine): implement compute_all_kpi master function
</commit_message>
<xml_diff>
--- a/supplynode/data/sample_data.xlsx
+++ b/supplynode/data/sample_data.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="suppliers" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sales_history" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="suppliers" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="sales_history" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,9 +18,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -51,9 +50,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,6 +508,11 @@
           <t>active</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>opening_stock</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -571,12 +576,15 @@
           <t>Kochi-WH01</t>
         </is>
       </c>
-      <c r="P2" s="1" t="n">
+      <c r="P2" s="2" t="n">
         <v>46228</v>
       </c>
       <c r="Q2" t="b">
         <v>1</v>
       </c>
+      <c r="R2" t="n">
+        <v>1550</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -640,12 +648,15 @@
           <t>Kochi-WH01</t>
         </is>
       </c>
-      <c r="P3" s="1" t="n">
+      <c r="P3" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="Q3" t="b">
         <v>1</v>
       </c>
+      <c r="R3" t="n">
+        <v>1250</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -709,12 +720,15 @@
           <t>Kochi-WH01</t>
         </is>
       </c>
-      <c r="P4" s="1" t="n">
+      <c r="P4" s="2" t="n">
         <v>46221</v>
       </c>
       <c r="Q4" t="b">
         <v>1</v>
       </c>
+      <c r="R4" t="n">
+        <v>410</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -778,12 +792,15 @@
           <t>Kochi-WH01</t>
         </is>
       </c>
-      <c r="P5" s="1" t="n">
+      <c r="P5" s="2" t="n">
         <v>46231</v>
       </c>
       <c r="Q5" t="b">
         <v>1</v>
       </c>
+      <c r="R5" t="n">
+        <v>270</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -847,11 +864,14 @@
           <t>Kochi-WH01</t>
         </is>
       </c>
-      <c r="P6" s="1" t="n">
+      <c r="P6" s="2" t="n">
         <v>46233</v>
       </c>
       <c r="Q6" t="b">
         <v>1</v>
+      </c>
+      <c r="R6" t="n">
+        <v>2400</v>
       </c>
     </row>
   </sheetData>
@@ -1158,7 +1178,7 @@
           <t>TXN0001</t>
         </is>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B2" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -1198,7 +1218,7 @@
           <t>TXN0002</t>
         </is>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1238,7 +1258,7 @@
           <t>TXN0003</t>
         </is>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -1278,7 +1298,7 @@
           <t>TXN0004</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -1318,7 +1338,7 @@
           <t>TXN0005</t>
         </is>
       </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -1358,7 +1378,7 @@
           <t>TXN0006</t>
         </is>
       </c>
-      <c r="B7" s="1" t="n">
+      <c r="B7" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -1398,7 +1418,7 @@
           <t>TXN0007</t>
         </is>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -1438,7 +1458,7 @@
           <t>TXN0008</t>
         </is>
       </c>
-      <c r="B9" s="1" t="n">
+      <c r="B9" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -1478,7 +1498,7 @@
           <t>TXN0009</t>
         </is>
       </c>
-      <c r="B10" s="1" t="n">
+      <c r="B10" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -1518,7 +1538,7 @@
           <t>TXN0010</t>
         </is>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B11" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -1558,7 +1578,7 @@
           <t>TXN0011</t>
         </is>
       </c>
-      <c r="B12" s="1" t="n">
+      <c r="B12" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -1598,7 +1618,7 @@
           <t>TXN0012</t>
         </is>
       </c>
-      <c r="B13" s="1" t="n">
+      <c r="B13" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -1638,7 +1658,7 @@
           <t>TXN0013</t>
         </is>
       </c>
-      <c r="B14" s="1" t="n">
+      <c r="B14" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="C14" t="inlineStr">
@@ -1678,7 +1698,7 @@
           <t>TXN0014</t>
         </is>
       </c>
-      <c r="B15" s="1" t="n">
+      <c r="B15" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="C15" t="inlineStr">
@@ -1718,7 +1738,7 @@
           <t>TXN0015</t>
         </is>
       </c>
-      <c r="B16" s="1" t="n">
+      <c r="B16" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="C16" t="inlineStr">
@@ -1758,7 +1778,7 @@
           <t>TXN0016</t>
         </is>
       </c>
-      <c r="B17" s="1" t="n">
+      <c r="B17" s="2" t="n">
         <v>46207</v>
       </c>
       <c r="C17" t="inlineStr">
@@ -1798,7 +1818,7 @@
           <t>TXN0017</t>
         </is>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B18" s="2" t="n">
         <v>46207</v>
       </c>
       <c r="C18" t="inlineStr">
@@ -1838,7 +1858,7 @@
           <t>TXN0018</t>
         </is>
       </c>
-      <c r="B19" s="1" t="n">
+      <c r="B19" s="2" t="n">
         <v>46207</v>
       </c>
       <c r="C19" t="inlineStr">
@@ -1878,7 +1898,7 @@
           <t>TXN0019</t>
         </is>
       </c>
-      <c r="B20" s="1" t="n">
+      <c r="B20" s="2" t="n">
         <v>46207</v>
       </c>
       <c r="C20" t="inlineStr">
@@ -1918,7 +1938,7 @@
           <t>TXN0020</t>
         </is>
       </c>
-      <c r="B21" s="1" t="n">
+      <c r="B21" s="2" t="n">
         <v>46207</v>
       </c>
       <c r="C21" t="inlineStr">
@@ -1958,7 +1978,7 @@
           <t>TXN0021</t>
         </is>
       </c>
-      <c r="B22" s="1" t="n">
+      <c r="B22" s="2" t="n">
         <v>46208</v>
       </c>
       <c r="C22" t="inlineStr">
@@ -1998,7 +2018,7 @@
           <t>TXN0022</t>
         </is>
       </c>
-      <c r="B23" s="1" t="n">
+      <c r="B23" s="2" t="n">
         <v>46208</v>
       </c>
       <c r="C23" t="inlineStr">
@@ -2038,7 +2058,7 @@
           <t>TXN0023</t>
         </is>
       </c>
-      <c r="B24" s="1" t="n">
+      <c r="B24" s="2" t="n">
         <v>46208</v>
       </c>
       <c r="C24" t="inlineStr">
@@ -2078,7 +2098,7 @@
           <t>TXN0024</t>
         </is>
       </c>
-      <c r="B25" s="1" t="n">
+      <c r="B25" s="2" t="n">
         <v>46208</v>
       </c>
       <c r="C25" t="inlineStr">
@@ -2118,7 +2138,7 @@
           <t>TXN0025</t>
         </is>
       </c>
-      <c r="B26" s="1" t="n">
+      <c r="B26" s="2" t="n">
         <v>46208</v>
       </c>
       <c r="C26" t="inlineStr">
@@ -2158,7 +2178,7 @@
           <t>TXN0026</t>
         </is>
       </c>
-      <c r="B27" s="1" t="n">
+      <c r="B27" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="C27" t="inlineStr">
@@ -2198,7 +2218,7 @@
           <t>TXN0027</t>
         </is>
       </c>
-      <c r="B28" s="1" t="n">
+      <c r="B28" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="C28" t="inlineStr">
@@ -2238,7 +2258,7 @@
           <t>TXN0028</t>
         </is>
       </c>
-      <c r="B29" s="1" t="n">
+      <c r="B29" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="C29" t="inlineStr">
@@ -2278,7 +2298,7 @@
           <t>TXN0029</t>
         </is>
       </c>
-      <c r="B30" s="1" t="n">
+      <c r="B30" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="C30" t="inlineStr">
@@ -2318,7 +2338,7 @@
           <t>TXN0030</t>
         </is>
       </c>
-      <c r="B31" s="1" t="n">
+      <c r="B31" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="C31" t="inlineStr">
@@ -2358,7 +2378,7 @@
           <t>TXN0031</t>
         </is>
       </c>
-      <c r="B32" s="1" t="n">
+      <c r="B32" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="C32" t="inlineStr">
@@ -2398,7 +2418,7 @@
           <t>TXN0032</t>
         </is>
       </c>
-      <c r="B33" s="1" t="n">
+      <c r="B33" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="C33" t="inlineStr">
@@ -2438,7 +2458,7 @@
           <t>TXN0033</t>
         </is>
       </c>
-      <c r="B34" s="1" t="n">
+      <c r="B34" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="C34" t="inlineStr">
@@ -2478,7 +2498,7 @@
           <t>TXN0034</t>
         </is>
       </c>
-      <c r="B35" s="1" t="n">
+      <c r="B35" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="C35" t="inlineStr">
@@ -2518,7 +2538,7 @@
           <t>TXN0035</t>
         </is>
       </c>
-      <c r="B36" s="1" t="n">
+      <c r="B36" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="C36" t="inlineStr">
@@ -2558,7 +2578,7 @@
           <t>TXN0036</t>
         </is>
       </c>
-      <c r="B37" s="1" t="n">
+      <c r="B37" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="C37" t="inlineStr">
@@ -2598,7 +2618,7 @@
           <t>TXN0037</t>
         </is>
       </c>
-      <c r="B38" s="1" t="n">
+      <c r="B38" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="C38" t="inlineStr">
@@ -2638,7 +2658,7 @@
           <t>TXN0038</t>
         </is>
       </c>
-      <c r="B39" s="1" t="n">
+      <c r="B39" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="C39" t="inlineStr">
@@ -2678,7 +2698,7 @@
           <t>TXN0039</t>
         </is>
       </c>
-      <c r="B40" s="1" t="n">
+      <c r="B40" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="C40" t="inlineStr">
@@ -2718,7 +2738,7 @@
           <t>TXN0040</t>
         </is>
       </c>
-      <c r="B41" s="1" t="n">
+      <c r="B41" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="C41" t="inlineStr">
@@ -2758,7 +2778,7 @@
           <t>TXN0041</t>
         </is>
       </c>
-      <c r="B42" s="1" t="n">
+      <c r="B42" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="C42" t="inlineStr">
@@ -2798,7 +2818,7 @@
           <t>TXN0042</t>
         </is>
       </c>
-      <c r="B43" s="1" t="n">
+      <c r="B43" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="C43" t="inlineStr">
@@ -2838,7 +2858,7 @@
           <t>TXN0043</t>
         </is>
       </c>
-      <c r="B44" s="1" t="n">
+      <c r="B44" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="C44" t="inlineStr">
@@ -2878,7 +2898,7 @@
           <t>TXN0044</t>
         </is>
       </c>
-      <c r="B45" s="1" t="n">
+      <c r="B45" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="C45" t="inlineStr">
@@ -2918,7 +2938,7 @@
           <t>TXN0045</t>
         </is>
       </c>
-      <c r="B46" s="1" t="n">
+      <c r="B46" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="C46" t="inlineStr">
@@ -2958,7 +2978,7 @@
           <t>TXN0046</t>
         </is>
       </c>
-      <c r="B47" s="1" t="n">
+      <c r="B47" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="C47" t="inlineStr">
@@ -2998,7 +3018,7 @@
           <t>TXN0047</t>
         </is>
       </c>
-      <c r="B48" s="1" t="n">
+      <c r="B48" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="C48" t="inlineStr">
@@ -3038,7 +3058,7 @@
           <t>TXN0048</t>
         </is>
       </c>
-      <c r="B49" s="1" t="n">
+      <c r="B49" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="C49" t="inlineStr">
@@ -3078,7 +3098,7 @@
           <t>TXN0049</t>
         </is>
       </c>
-      <c r="B50" s="1" t="n">
+      <c r="B50" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="C50" t="inlineStr">
@@ -3118,7 +3138,7 @@
           <t>TXN0050</t>
         </is>
       </c>
-      <c r="B51" s="1" t="n">
+      <c r="B51" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="C51" t="inlineStr">
@@ -3158,7 +3178,7 @@
           <t>TXN0051</t>
         </is>
       </c>
-      <c r="B52" s="1" t="n">
+      <c r="B52" s="2" t="n">
         <v>46214</v>
       </c>
       <c r="C52" t="inlineStr">
@@ -3198,7 +3218,7 @@
           <t>TXN0052</t>
         </is>
       </c>
-      <c r="B53" s="1" t="n">
+      <c r="B53" s="2" t="n">
         <v>46214</v>
       </c>
       <c r="C53" t="inlineStr">
@@ -3238,7 +3258,7 @@
           <t>TXN0053</t>
         </is>
       </c>
-      <c r="B54" s="1" t="n">
+      <c r="B54" s="2" t="n">
         <v>46214</v>
       </c>
       <c r="C54" t="inlineStr">
@@ -3278,7 +3298,7 @@
           <t>TXN0054</t>
         </is>
       </c>
-      <c r="B55" s="1" t="n">
+      <c r="B55" s="2" t="n">
         <v>46214</v>
       </c>
       <c r="C55" t="inlineStr">
@@ -3318,7 +3338,7 @@
           <t>TXN0055</t>
         </is>
       </c>
-      <c r="B56" s="1" t="n">
+      <c r="B56" s="2" t="n">
         <v>46214</v>
       </c>
       <c r="C56" t="inlineStr">
@@ -3358,7 +3378,7 @@
           <t>TXN0056</t>
         </is>
       </c>
-      <c r="B57" s="1" t="n">
+      <c r="B57" s="2" t="n">
         <v>46215</v>
       </c>
       <c r="C57" t="inlineStr">
@@ -3398,7 +3418,7 @@
           <t>TXN0057</t>
         </is>
       </c>
-      <c r="B58" s="1" t="n">
+      <c r="B58" s="2" t="n">
         <v>46215</v>
       </c>
       <c r="C58" t="inlineStr">
@@ -3438,7 +3458,7 @@
           <t>TXN0058</t>
         </is>
       </c>
-      <c r="B59" s="1" t="n">
+      <c r="B59" s="2" t="n">
         <v>46215</v>
       </c>
       <c r="C59" t="inlineStr">
@@ -3478,7 +3498,7 @@
           <t>TXN0059</t>
         </is>
       </c>
-      <c r="B60" s="1" t="n">
+      <c r="B60" s="2" t="n">
         <v>46215</v>
       </c>
       <c r="C60" t="inlineStr">
@@ -3518,7 +3538,7 @@
           <t>TXN0060</t>
         </is>
       </c>
-      <c r="B61" s="1" t="n">
+      <c r="B61" s="2" t="n">
         <v>46215</v>
       </c>
       <c r="C61" t="inlineStr">
@@ -3558,7 +3578,7 @@
           <t>TXN0061</t>
         </is>
       </c>
-      <c r="B62" s="1" t="n">
+      <c r="B62" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="C62" t="inlineStr">
@@ -3598,7 +3618,7 @@
           <t>TXN0062</t>
         </is>
       </c>
-      <c r="B63" s="1" t="n">
+      <c r="B63" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="C63" t="inlineStr">
@@ -3638,7 +3658,7 @@
           <t>TXN0063</t>
         </is>
       </c>
-      <c r="B64" s="1" t="n">
+      <c r="B64" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="C64" t="inlineStr">
@@ -3678,7 +3698,7 @@
           <t>TXN0064</t>
         </is>
       </c>
-      <c r="B65" s="1" t="n">
+      <c r="B65" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="C65" t="inlineStr">
@@ -3718,7 +3738,7 @@
           <t>TXN0065</t>
         </is>
       </c>
-      <c r="B66" s="1" t="n">
+      <c r="B66" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="C66" t="inlineStr">
@@ -3758,7 +3778,7 @@
           <t>TXN0066</t>
         </is>
       </c>
-      <c r="B67" s="1" t="n">
+      <c r="B67" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="C67" t="inlineStr">
@@ -3798,7 +3818,7 @@
           <t>TXN0067</t>
         </is>
       </c>
-      <c r="B68" s="1" t="n">
+      <c r="B68" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="C68" t="inlineStr">
@@ -3838,7 +3858,7 @@
           <t>TXN0068</t>
         </is>
       </c>
-      <c r="B69" s="1" t="n">
+      <c r="B69" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="C69" t="inlineStr">
@@ -3878,7 +3898,7 @@
           <t>TXN0069</t>
         </is>
       </c>
-      <c r="B70" s="1" t="n">
+      <c r="B70" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="C70" t="inlineStr">
@@ -3918,7 +3938,7 @@
           <t>TXN0070</t>
         </is>
       </c>
-      <c r="B71" s="1" t="n">
+      <c r="B71" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="C71" t="inlineStr">
@@ -3958,7 +3978,7 @@
           <t>TXN0071</t>
         </is>
       </c>
-      <c r="B72" s="1" t="n">
+      <c r="B72" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="C72" t="inlineStr">
@@ -3998,7 +4018,7 @@
           <t>TXN0072</t>
         </is>
       </c>
-      <c r="B73" s="1" t="n">
+      <c r="B73" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="C73" t="inlineStr">
@@ -4038,7 +4058,7 @@
           <t>TXN0073</t>
         </is>
       </c>
-      <c r="B74" s="1" t="n">
+      <c r="B74" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="C74" t="inlineStr">
@@ -4078,7 +4098,7 @@
           <t>TXN0074</t>
         </is>
       </c>
-      <c r="B75" s="1" t="n">
+      <c r="B75" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="C75" t="inlineStr">
@@ -4118,7 +4138,7 @@
           <t>TXN0075</t>
         </is>
       </c>
-      <c r="B76" s="1" t="n">
+      <c r="B76" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="C76" t="inlineStr">
@@ -4158,7 +4178,7 @@
           <t>TXN0076</t>
         </is>
       </c>
-      <c r="B77" s="1" t="n">
+      <c r="B77" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="C77" t="inlineStr">
@@ -4198,7 +4218,7 @@
           <t>TXN0077</t>
         </is>
       </c>
-      <c r="B78" s="1" t="n">
+      <c r="B78" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="C78" t="inlineStr">
@@ -4238,7 +4258,7 @@
           <t>TXN0078</t>
         </is>
       </c>
-      <c r="B79" s="1" t="n">
+      <c r="B79" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="C79" t="inlineStr">
@@ -4278,7 +4298,7 @@
           <t>TXN0079</t>
         </is>
       </c>
-      <c r="B80" s="1" t="n">
+      <c r="B80" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="C80" t="inlineStr">
@@ -4318,7 +4338,7 @@
           <t>TXN0080</t>
         </is>
       </c>
-      <c r="B81" s="1" t="n">
+      <c r="B81" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="C81" t="inlineStr">
@@ -4358,7 +4378,7 @@
           <t>TXN0081</t>
         </is>
       </c>
-      <c r="B82" s="1" t="n">
+      <c r="B82" s="2" t="n">
         <v>46220</v>
       </c>
       <c r="C82" t="inlineStr">
@@ -4398,7 +4418,7 @@
           <t>TXN0082</t>
         </is>
       </c>
-      <c r="B83" s="1" t="n">
+      <c r="B83" s="2" t="n">
         <v>46220</v>
       </c>
       <c r="C83" t="inlineStr">
@@ -4438,7 +4458,7 @@
           <t>TXN0083</t>
         </is>
       </c>
-      <c r="B84" s="1" t="n">
+      <c r="B84" s="2" t="n">
         <v>46220</v>
       </c>
       <c r="C84" t="inlineStr">
@@ -4478,7 +4498,7 @@
           <t>TXN0084</t>
         </is>
       </c>
-      <c r="B85" s="1" t="n">
+      <c r="B85" s="2" t="n">
         <v>46220</v>
       </c>
       <c r="C85" t="inlineStr">
@@ -4518,7 +4538,7 @@
           <t>TXN0085</t>
         </is>
       </c>
-      <c r="B86" s="1" t="n">
+      <c r="B86" s="2" t="n">
         <v>46220</v>
       </c>
       <c r="C86" t="inlineStr">
@@ -4558,7 +4578,7 @@
           <t>TXN0086</t>
         </is>
       </c>
-      <c r="B87" s="1" t="n">
+      <c r="B87" s="2" t="n">
         <v>46221</v>
       </c>
       <c r="C87" t="inlineStr">
@@ -4598,7 +4618,7 @@
           <t>TXN0087</t>
         </is>
       </c>
-      <c r="B88" s="1" t="n">
+      <c r="B88" s="2" t="n">
         <v>46221</v>
       </c>
       <c r="C88" t="inlineStr">
@@ -4638,7 +4658,7 @@
           <t>TXN0088</t>
         </is>
       </c>
-      <c r="B89" s="1" t="n">
+      <c r="B89" s="2" t="n">
         <v>46221</v>
       </c>
       <c r="C89" t="inlineStr">
@@ -4678,7 +4698,7 @@
           <t>TXN0089</t>
         </is>
       </c>
-      <c r="B90" s="1" t="n">
+      <c r="B90" s="2" t="n">
         <v>46221</v>
       </c>
       <c r="C90" t="inlineStr">
@@ -4718,7 +4738,7 @@
           <t>TXN0090</t>
         </is>
       </c>
-      <c r="B91" s="1" t="n">
+      <c r="B91" s="2" t="n">
         <v>46221</v>
       </c>
       <c r="C91" t="inlineStr">
@@ -4758,7 +4778,7 @@
           <t>TXN0091</t>
         </is>
       </c>
-      <c r="B92" s="1" t="n">
+      <c r="B92" s="2" t="n">
         <v>46222</v>
       </c>
       <c r="C92" t="inlineStr">
@@ -4798,7 +4818,7 @@
           <t>TXN0092</t>
         </is>
       </c>
-      <c r="B93" s="1" t="n">
+      <c r="B93" s="2" t="n">
         <v>46222</v>
       </c>
       <c r="C93" t="inlineStr">
@@ -4838,7 +4858,7 @@
           <t>TXN0093</t>
         </is>
       </c>
-      <c r="B94" s="1" t="n">
+      <c r="B94" s="2" t="n">
         <v>46222</v>
       </c>
       <c r="C94" t="inlineStr">
@@ -4878,7 +4898,7 @@
           <t>TXN0094</t>
         </is>
       </c>
-      <c r="B95" s="1" t="n">
+      <c r="B95" s="2" t="n">
         <v>46222</v>
       </c>
       <c r="C95" t="inlineStr">
@@ -4918,7 +4938,7 @@
           <t>TXN0095</t>
         </is>
       </c>
-      <c r="B96" s="1" t="n">
+      <c r="B96" s="2" t="n">
         <v>46222</v>
       </c>
       <c r="C96" t="inlineStr">
@@ -4958,7 +4978,7 @@
           <t>TXN0096</t>
         </is>
       </c>
-      <c r="B97" s="1" t="n">
+      <c r="B97" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="C97" t="inlineStr">
@@ -4998,7 +5018,7 @@
           <t>TXN0097</t>
         </is>
       </c>
-      <c r="B98" s="1" t="n">
+      <c r="B98" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="C98" t="inlineStr">
@@ -5038,7 +5058,7 @@
           <t>TXN0098</t>
         </is>
       </c>
-      <c r="B99" s="1" t="n">
+      <c r="B99" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="C99" t="inlineStr">
@@ -5078,7 +5098,7 @@
           <t>TXN0099</t>
         </is>
       </c>
-      <c r="B100" s="1" t="n">
+      <c r="B100" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="C100" t="inlineStr">
@@ -5118,7 +5138,7 @@
           <t>TXN0100</t>
         </is>
       </c>
-      <c r="B101" s="1" t="n">
+      <c r="B101" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="C101" t="inlineStr">
@@ -5158,7 +5178,7 @@
           <t>TXN0101</t>
         </is>
       </c>
-      <c r="B102" s="1" t="n">
+      <c r="B102" s="2" t="n">
         <v>46224</v>
       </c>
       <c r="C102" t="inlineStr">
@@ -5198,7 +5218,7 @@
           <t>TXN0102</t>
         </is>
       </c>
-      <c r="B103" s="1" t="n">
+      <c r="B103" s="2" t="n">
         <v>46224</v>
       </c>
       <c r="C103" t="inlineStr">
@@ -5238,7 +5258,7 @@
           <t>TXN0103</t>
         </is>
       </c>
-      <c r="B104" s="1" t="n">
+      <c r="B104" s="2" t="n">
         <v>46224</v>
       </c>
       <c r="C104" t="inlineStr">
@@ -5278,7 +5298,7 @@
           <t>TXN0104</t>
         </is>
       </c>
-      <c r="B105" s="1" t="n">
+      <c r="B105" s="2" t="n">
         <v>46224</v>
       </c>
       <c r="C105" t="inlineStr">
@@ -5318,7 +5338,7 @@
           <t>TXN0105</t>
         </is>
       </c>
-      <c r="B106" s="1" t="n">
+      <c r="B106" s="2" t="n">
         <v>46224</v>
       </c>
       <c r="C106" t="inlineStr">
@@ -5358,7 +5378,7 @@
           <t>TXN0106</t>
         </is>
       </c>
-      <c r="B107" s="1" t="n">
+      <c r="B107" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="C107" t="inlineStr">
@@ -5398,7 +5418,7 @@
           <t>TXN0107</t>
         </is>
       </c>
-      <c r="B108" s="1" t="n">
+      <c r="B108" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="C108" t="inlineStr">
@@ -5438,7 +5458,7 @@
           <t>TXN0108</t>
         </is>
       </c>
-      <c r="B109" s="1" t="n">
+      <c r="B109" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="C109" t="inlineStr">
@@ -5478,7 +5498,7 @@
           <t>TXN0109</t>
         </is>
       </c>
-      <c r="B110" s="1" t="n">
+      <c r="B110" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="C110" t="inlineStr">
@@ -5518,7 +5538,7 @@
           <t>TXN0110</t>
         </is>
       </c>
-      <c r="B111" s="1" t="n">
+      <c r="B111" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="C111" t="inlineStr">
@@ -5558,7 +5578,7 @@
           <t>TXN0111</t>
         </is>
       </c>
-      <c r="B112" s="1" t="n">
+      <c r="B112" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="C112" t="inlineStr">
@@ -5598,7 +5618,7 @@
           <t>TXN0112</t>
         </is>
       </c>
-      <c r="B113" s="1" t="n">
+      <c r="B113" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="C113" t="inlineStr">
@@ -5638,7 +5658,7 @@
           <t>TXN0113</t>
         </is>
       </c>
-      <c r="B114" s="1" t="n">
+      <c r="B114" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="C114" t="inlineStr">
@@ -5678,7 +5698,7 @@
           <t>TXN0114</t>
         </is>
       </c>
-      <c r="B115" s="1" t="n">
+      <c r="B115" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="C115" t="inlineStr">
@@ -5718,7 +5738,7 @@
           <t>TXN0115</t>
         </is>
       </c>
-      <c r="B116" s="1" t="n">
+      <c r="B116" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="C116" t="inlineStr">
@@ -5758,7 +5778,7 @@
           <t>TXN0116</t>
         </is>
       </c>
-      <c r="B117" s="1" t="n">
+      <c r="B117" s="2" t="n">
         <v>46227</v>
       </c>
       <c r="C117" t="inlineStr">
@@ -5798,7 +5818,7 @@
           <t>TXN0117</t>
         </is>
       </c>
-      <c r="B118" s="1" t="n">
+      <c r="B118" s="2" t="n">
         <v>46227</v>
       </c>
       <c r="C118" t="inlineStr">
@@ -5838,7 +5858,7 @@
           <t>TXN0118</t>
         </is>
       </c>
-      <c r="B119" s="1" t="n">
+      <c r="B119" s="2" t="n">
         <v>46227</v>
       </c>
       <c r="C119" t="inlineStr">
@@ -5878,7 +5898,7 @@
           <t>TXN0119</t>
         </is>
       </c>
-      <c r="B120" s="1" t="n">
+      <c r="B120" s="2" t="n">
         <v>46227</v>
       </c>
       <c r="C120" t="inlineStr">
@@ -5918,7 +5938,7 @@
           <t>TXN0120</t>
         </is>
       </c>
-      <c r="B121" s="1" t="n">
+      <c r="B121" s="2" t="n">
         <v>46227</v>
       </c>
       <c r="C121" t="inlineStr">
@@ -5958,7 +5978,7 @@
           <t>TXN0121</t>
         </is>
       </c>
-      <c r="B122" s="1" t="n">
+      <c r="B122" s="2" t="n">
         <v>46228</v>
       </c>
       <c r="C122" t="inlineStr">
@@ -5998,7 +6018,7 @@
           <t>TXN0122</t>
         </is>
       </c>
-      <c r="B123" s="1" t="n">
+      <c r="B123" s="2" t="n">
         <v>46228</v>
       </c>
       <c r="C123" t="inlineStr">
@@ -6038,7 +6058,7 @@
           <t>TXN0123</t>
         </is>
       </c>
-      <c r="B124" s="1" t="n">
+      <c r="B124" s="2" t="n">
         <v>46228</v>
       </c>
       <c r="C124" t="inlineStr">
@@ -6078,7 +6098,7 @@
           <t>TXN0124</t>
         </is>
       </c>
-      <c r="B125" s="1" t="n">
+      <c r="B125" s="2" t="n">
         <v>46228</v>
       </c>
       <c r="C125" t="inlineStr">
@@ -6118,7 +6138,7 @@
           <t>TXN0125</t>
         </is>
       </c>
-      <c r="B126" s="1" t="n">
+      <c r="B126" s="2" t="n">
         <v>46228</v>
       </c>
       <c r="C126" t="inlineStr">
@@ -6158,7 +6178,7 @@
           <t>TXN0126</t>
         </is>
       </c>
-      <c r="B127" s="1" t="n">
+      <c r="B127" s="2" t="n">
         <v>46229</v>
       </c>
       <c r="C127" t="inlineStr">
@@ -6198,7 +6218,7 @@
           <t>TXN0127</t>
         </is>
       </c>
-      <c r="B128" s="1" t="n">
+      <c r="B128" s="2" t="n">
         <v>46229</v>
       </c>
       <c r="C128" t="inlineStr">
@@ -6238,7 +6258,7 @@
           <t>TXN0128</t>
         </is>
       </c>
-      <c r="B129" s="1" t="n">
+      <c r="B129" s="2" t="n">
         <v>46229</v>
       </c>
       <c r="C129" t="inlineStr">
@@ -6278,7 +6298,7 @@
           <t>TXN0129</t>
         </is>
       </c>
-      <c r="B130" s="1" t="n">
+      <c r="B130" s="2" t="n">
         <v>46229</v>
       </c>
       <c r="C130" t="inlineStr">
@@ -6318,7 +6338,7 @@
           <t>TXN0130</t>
         </is>
       </c>
-      <c r="B131" s="1" t="n">
+      <c r="B131" s="2" t="n">
         <v>46229</v>
       </c>
       <c r="C131" t="inlineStr">
@@ -6358,7 +6378,7 @@
           <t>TXN0131</t>
         </is>
       </c>
-      <c r="B132" s="1" t="n">
+      <c r="B132" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="C132" t="inlineStr">
@@ -6398,7 +6418,7 @@
           <t>TXN0132</t>
         </is>
       </c>
-      <c r="B133" s="1" t="n">
+      <c r="B133" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="C133" t="inlineStr">
@@ -6438,7 +6458,7 @@
           <t>TXN0133</t>
         </is>
       </c>
-      <c r="B134" s="1" t="n">
+      <c r="B134" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="C134" t="inlineStr">
@@ -6478,7 +6498,7 @@
           <t>TXN0134</t>
         </is>
       </c>
-      <c r="B135" s="1" t="n">
+      <c r="B135" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="C135" t="inlineStr">
@@ -6518,7 +6538,7 @@
           <t>TXN0135</t>
         </is>
       </c>
-      <c r="B136" s="1" t="n">
+      <c r="B136" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="C136" t="inlineStr">
@@ -6558,7 +6578,7 @@
           <t>TXN0136</t>
         </is>
       </c>
-      <c r="B137" s="1" t="n">
+      <c r="B137" s="2" t="n">
         <v>46231</v>
       </c>
       <c r="C137" t="inlineStr">
@@ -6598,7 +6618,7 @@
           <t>TXN0137</t>
         </is>
       </c>
-      <c r="B138" s="1" t="n">
+      <c r="B138" s="2" t="n">
         <v>46231</v>
       </c>
       <c r="C138" t="inlineStr">
@@ -6638,7 +6658,7 @@
           <t>TXN0138</t>
         </is>
       </c>
-      <c r="B139" s="1" t="n">
+      <c r="B139" s="2" t="n">
         <v>46231</v>
       </c>
       <c r="C139" t="inlineStr">
@@ -6678,7 +6698,7 @@
           <t>TXN0139</t>
         </is>
       </c>
-      <c r="B140" s="1" t="n">
+      <c r="B140" s="2" t="n">
         <v>46231</v>
       </c>
       <c r="C140" t="inlineStr">
@@ -6718,7 +6738,7 @@
           <t>TXN0140</t>
         </is>
       </c>
-      <c r="B141" s="1" t="n">
+      <c r="B141" s="2" t="n">
         <v>46231</v>
       </c>
       <c r="C141" t="inlineStr">
@@ -6758,7 +6778,7 @@
           <t>TXN0141</t>
         </is>
       </c>
-      <c r="B142" s="1" t="n">
+      <c r="B142" s="2" t="n">
         <v>46232</v>
       </c>
       <c r="C142" t="inlineStr">
@@ -6798,7 +6818,7 @@
           <t>TXN0142</t>
         </is>
       </c>
-      <c r="B143" s="1" t="n">
+      <c r="B143" s="2" t="n">
         <v>46232</v>
       </c>
       <c r="C143" t="inlineStr">
@@ -6838,7 +6858,7 @@
           <t>TXN0143</t>
         </is>
       </c>
-      <c r="B144" s="1" t="n">
+      <c r="B144" s="2" t="n">
         <v>46232</v>
       </c>
       <c r="C144" t="inlineStr">
@@ -6878,7 +6898,7 @@
           <t>TXN0144</t>
         </is>
       </c>
-      <c r="B145" s="1" t="n">
+      <c r="B145" s="2" t="n">
         <v>46232</v>
       </c>
       <c r="C145" t="inlineStr">
@@ -6918,7 +6938,7 @@
           <t>TXN0145</t>
         </is>
       </c>
-      <c r="B146" s="1" t="n">
+      <c r="B146" s="2" t="n">
         <v>46232</v>
       </c>
       <c r="C146" t="inlineStr">
@@ -6958,7 +6978,7 @@
           <t>TXN0146</t>
         </is>
       </c>
-      <c r="B147" s="1" t="n">
+      <c r="B147" s="2" t="n">
         <v>46233</v>
       </c>
       <c r="C147" t="inlineStr">
@@ -6998,7 +7018,7 @@
           <t>TXN0147</t>
         </is>
       </c>
-      <c r="B148" s="1" t="n">
+      <c r="B148" s="2" t="n">
         <v>46233</v>
       </c>
       <c r="C148" t="inlineStr">
@@ -7038,7 +7058,7 @@
           <t>TXN0148</t>
         </is>
       </c>
-      <c r="B149" s="1" t="n">
+      <c r="B149" s="2" t="n">
         <v>46233</v>
       </c>
       <c r="C149" t="inlineStr">
@@ -7078,7 +7098,7 @@
           <t>TXN0149</t>
         </is>
       </c>
-      <c r="B150" s="1" t="n">
+      <c r="B150" s="2" t="n">
         <v>46233</v>
       </c>
       <c r="C150" t="inlineStr">
@@ -7118,7 +7138,7 @@
           <t>TXN0150</t>
         </is>
       </c>
-      <c r="B151" s="1" t="n">
+      <c r="B151" s="2" t="n">
         <v>46233</v>
       </c>
       <c r="C151" t="inlineStr">

</xml_diff>